<commit_message>
Add download_all_scraped_pdfs script and upload 43 downloaded scraped PDF documents
</commit_message>
<xml_diff>
--- a/scraped_results/sikkim_policy_files_index.xlsx
+++ b/scraped_results/sikkim_policy_files_index.xlsx
@@ -8300,12 +8300,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="110" customWidth="1" min="2" max="2"/>
-    <col width="85" customWidth="1" min="3" max="3"/>
+    <col width="112" customWidth="1" min="2" max="2"/>
+    <col width="88" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
@@ -8361,12 +8361,12 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>sikkim_policy_briefs/food and agriculture policies.pdf</t>
+          <t>sikkim_policy_briefs/Sikkim - consolidated policies.pdf</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>food and agriculture policies</t>
+          <t>Sikkim - consolidated policies</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
@@ -8381,7 +8381,7 @@
       </c>
       <c r="F2" s="6" t="inlineStr">
         <is>
-          <t>1.92 MB</t>
+          <t>7.14 MB</t>
         </is>
       </c>
       <c r="G2" s="6" t="inlineStr">
@@ -8401,12 +8401,12 @@
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>sikkim_policy_briefs/Sikkim - consolidated policies.pdf</t>
+          <t>sikkim_policy_briefs/Sikkim Green Policy _ A Policy Brief _ O.P. Jindal Global University.pdf</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
-          <t>Sikkim - consolidated policies</t>
+          <t>Sikkim Green Policy _ A Policy Brief _ O.P. Jindal Global University</t>
         </is>
       </c>
       <c r="D3" s="8" t="inlineStr">
@@ -8421,12 +8421,12 @@
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>7.14 MB</t>
+          <t>757.73 KB</t>
         </is>
       </c>
       <c r="G3" s="9" t="inlineStr">
         <is>
-          <t>2026-05-19 12:13</t>
+          <t>2026-05-19 11:45</t>
         </is>
       </c>
       <c r="H3" s="8" t="inlineStr">
@@ -8441,12 +8441,12 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>sikkim_policy_briefs/Sikkim Green Policy _ A Policy Brief _ O.P. Jindal Global University.pdf</t>
+          <t>sikkim_policy_briefs/Sikkim Policies.pdf</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Sikkim Green Policy _ A Policy Brief _ O.P. Jindal Global University</t>
+          <t>Sikkim Policies</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
@@ -8461,12 +8461,12 @@
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>757.73 KB</t>
+          <t>4.35 MB</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>2026-05-19 11:45</t>
+          <t>2026-05-19 12:04</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
@@ -8481,12 +8481,12 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>sikkim_policy_briefs/Sikkim Policies.pdf</t>
+          <t>sikkim_policy_briefs/World Bank Document Policies.pdf</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>Sikkim Policies</t>
+          <t>World Bank Document Policies</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
@@ -8501,12 +8501,12 @@
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
-          <t>4.35 MB</t>
+          <t>159.13 KB</t>
         </is>
       </c>
       <c r="G5" s="9" t="inlineStr">
         <is>
-          <t>2026-05-19 12:04</t>
+          <t>2026-05-19 12:12</t>
         </is>
       </c>
       <c r="H5" s="8" t="inlineStr">
@@ -8521,12 +8521,12 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>sikkim_policy_briefs/sikkim sustainable development goals, policies and programmes for their attention.pdf</t>
+          <t>sikkim_policy_briefs/food and agriculture policies.pdf</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>sikkim sustainable development goals, policies and programmes for their attention</t>
+          <t>food and agriculture policies</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -8541,12 +8541,12 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>3.12 MB</t>
+          <t>1.92 MB</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>2026-05-19 12:04</t>
+          <t>2026-05-19 12:13</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
@@ -8561,12 +8561,12 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>sikkim_policy_briefs/World Bank Document Policies.pdf</t>
+          <t>sikkim_policy_briefs/sikkim sustainable development goals, policies and programmes for their attention.pdf</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>World Bank Document Policies</t>
+          <t>sikkim sustainable development goals, policies and programmes for their attention</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
@@ -8581,12 +8581,12 @@
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
-          <t>159.13 KB</t>
+          <t>3.12 MB</t>
         </is>
       </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
-          <t>2026-05-19 12:12</t>
+          <t>2026-05-19 12:04</t>
         </is>
       </c>
       <c r="H7" s="8" t="inlineStr">
@@ -8601,37 +8601,37 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>scraping.py</t>
+          <t>scraped_policy_pdfs/006_Economics ofOrganicCashCropsand FoodCropsinSikkim Comparative Study.pdf</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>scraping</t>
+          <t>006_Economics ofOrganicCashCropsand FoodCropsinSikkim Comparative Study</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Python Source Code</t>
+          <t>PDF Document</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>.py</t>
+          <t>.pdf</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>19.33 KB</t>
+          <t>9.12 MB</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>2026-05-19 12:58</t>
+          <t>2026-05-19 16:19</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>Project Root</t>
+          <t>scraped_policy_pdfs</t>
         </is>
       </c>
     </row>
@@ -8641,37 +8641,37 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>requirements.txt</t>
+          <t>scraped_policy_pdfs/008_SustainableTourismPlanning and Development A Study of Selectedtouristdestination.pdf</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>requirements</t>
+          <t>008_SustainableTourismPlanning and Development A Study of Selectedtouristdestination</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>Text Document</t>
+          <t>PDF Document</t>
         </is>
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>.txt</t>
+          <t>.pdf</t>
         </is>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t>737 B</t>
+          <t>5.58 MB</t>
         </is>
       </c>
       <c r="G9" s="9" t="inlineStr">
         <is>
-          <t>2026-05-19 12:55</t>
+          <t>2026-05-19 16:19</t>
         </is>
       </c>
       <c r="H9" s="8" t="inlineStr">
         <is>
-          <t>Project Root</t>
+          <t>scraped_policy_pdfs</t>
         </is>
       </c>
     </row>
@@ -8681,33 +8681,37 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>.gitignore</t>
+          <t>scraped_policy_pdfs/010_Ecotourism andSustainable Developmentin the Indian Himalayan Region A Case Study.pdf</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>.gitignore</t>
+          <t>010_Ecotourism andSustainable Developmentin the Indian Himalayan Region A Case Study</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Configuration File</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr"/>
+          <t>PDF Document</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>.pdf</t>
+        </is>
+      </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>53 B</t>
+          <t>48.30 KB</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>2026-05-19 14:08</t>
+          <t>2026-05-19 16:19</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>Project Root</t>
+          <t>scraped_policy_pdfs</t>
         </is>
       </c>
     </row>
@@ -8717,35 +8721,1751 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
+          <t>scraped_policy_pdfs/012_Impact ofEcotourismon Village Economy and Society InSikkim.pdf</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>012_Impact ofEcotourismon Village Economy and Society InSikkim</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>PDF Document</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>.pdf</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>8.14 MB</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:19</t>
+        </is>
+      </c>
+      <c r="H11" s="8" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs/013_Climate change inSikkim A synthesis.pdf</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>013_Climate change inSikkim A synthesis</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>PDF Document</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>.pdf</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>617.51 KB</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:19</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs/014_Climate Change initiatives insikkim.pdf</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>014_Climate Change initiatives insikkim</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>PDF Document</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>.pdf</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>3.04 MB</t>
+        </is>
+      </c>
+      <c r="G13" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:19</t>
+        </is>
+      </c>
+      <c r="H13" s="8" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs/015_Comparative Analysis of ClimatePoliciesin Kerala andSikkim Alignment with the IP.pdf</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>015_Comparative Analysis of ClimatePoliciesin Kerala andSikkim Alignment with the IP</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>PDF Document</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>.pdf</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>1.00 MB</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:19</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="7" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs/017_An analysis of past three decade weather phenomenon in the mid-hills ofSikkimand.pdf</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>017_An analysis of past three decade weather phenomenon in the mid-hills ofSikkimand</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>PDF Document</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>.pdf</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>1.62 MB</t>
+        </is>
+      </c>
+      <c r="G15" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:19</t>
+        </is>
+      </c>
+      <c r="H15" s="8" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs/019_Knowledge attitudes and perceptions of students towardbiodiversityconservation w.pdf</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>019_Knowledge attitudes and perceptions of students towardbiodiversityconservation w</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>PDF Document</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>.pdf</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>2.91 MB</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:19</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs/020_Corporate Social Responsibility and Sustainable Development inSikkim A Critical .pdf</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">020_Corporate Social Responsibility and Sustainable Development inSikkim A Critical </t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>PDF Document</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>.pdf</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>1.25 MB</t>
+        </is>
+      </c>
+      <c r="G17" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:19</t>
+        </is>
+      </c>
+      <c r="H17" s="8" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs/021_A Review of Education inSikkimwith Northeast India A journey towardsSDG-4.pdf</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>021_A Review of Education inSikkimwith Northeast India A journey towardsSDG-4</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>PDF Document</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>.pdf</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>662.18 KB</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:19</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="7" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs/022_Outcome Evaluation ofSikkimState Finances.pdf</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>022_Outcome Evaluation ofSikkimState Finances</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>PDF Document</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>.pdf</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t>3.59 MB</t>
+        </is>
+      </c>
+      <c r="G19" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:19</t>
+        </is>
+      </c>
+      <c r="H19" s="8" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs/023_ResponsibleTourisminitiatives towards sustainabletourismdevelopment A case study.pdf</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>023_ResponsibleTourisminitiatives towards sustainabletourismdevelopment A case study</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>PDF Document</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>.pdf</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>5.24 MB</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:19</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs/025_Community development andtourism TheSikkimexperience in the Eastern Himalayas.pdf</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>025_Community development andtourism TheSikkimexperience in the Eastern Himalayas</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>PDF Document</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>.pdf</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>110.59 KB</t>
+        </is>
+      </c>
+      <c r="G21" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:19</t>
+        </is>
+      </c>
+      <c r="H21" s="8" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs/027_SUSTAINABLE TREKKING PRACTICES FOR REDUCINGPLASTICWASTE IN FRAGILE HIMALAYAN ECO.pdf</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>027_SUSTAINABLE TREKKING PRACTICES FOR REDUCINGPLASTICWASTE IN FRAGILE HIMALAYAN ECO</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>PDF Document</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>.pdf</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>3.28 MB</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:19</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="7" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs/028_Voices in the Void; The Politics of Knowledge aroundHydropowerDevelopment inSikk.pdf</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>028_Voices in the Void; The Politics of Knowledge aroundHydropowerDevelopment inSikk</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>PDF Document</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>.pdf</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>4.39 MB</t>
+        </is>
+      </c>
+      <c r="G23" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:19</t>
+        </is>
+      </c>
+      <c r="H23" s="8" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs/029_Benefit Sharing Among Local Communities ofHydropowerProjects inSikkim.pdf</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>029_Benefit Sharing Among Local Communities ofHydropowerProjects inSikkim</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>PDF Document</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>.pdf</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>3.11 MB</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:19</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="7" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs/030_The TeestaHydro PowerProjects A Historical Analysis of the Protest Movement in N.pdf</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>030_The TeestaHydro PowerProjects A Historical Analysis of the Protest Movement in N</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>PDF Document</t>
+        </is>
+      </c>
+      <c r="E25" s="9" t="inlineStr">
+        <is>
+          <t>.pdf</t>
+        </is>
+      </c>
+      <c r="F25" s="9" t="inlineStr">
+        <is>
+          <t>3.37 MB</t>
+        </is>
+      </c>
+      <c r="G25" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:19</t>
+        </is>
+      </c>
+      <c r="H25" s="8" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs/031_GreenIP Regime and the Issues of Environment Protection in the State ofSikkim A .pdf</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">031_GreenIP Regime and the Issues of Environment Protection in the State ofSikkim A </t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>PDF Document</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>.pdf</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>49.64 KB</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:19</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="7" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs/033_FoodSecurity and Management inSikkim Role of Public Distribution System and Maha.pdf</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>033_FoodSecurity and Management inSikkim Role of Public Distribution System and Maha</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>PDF Document</t>
+        </is>
+      </c>
+      <c r="E27" s="9" t="inlineStr">
+        <is>
+          <t>.pdf</t>
+        </is>
+      </c>
+      <c r="F27" s="9" t="inlineStr">
+        <is>
+          <t>7.05 MB</t>
+        </is>
+      </c>
+      <c r="G27" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:19</t>
+        </is>
+      </c>
+      <c r="H27" s="8" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs/034_Sikkim Development report.pdf</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>034_Sikkim Development report</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>PDF Document</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>.pdf</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>1.30 MB</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:19</t>
+        </is>
+      </c>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="7" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs/035_Opportunities and challenges of the globally important traditional agriculture h.pdf</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>035_Opportunities and challenges of the globally important traditional agriculture h</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>PDF Document</t>
+        </is>
+      </c>
+      <c r="E29" s="9" t="inlineStr">
+        <is>
+          <t>.pdf</t>
+        </is>
+      </c>
+      <c r="F29" s="9" t="inlineStr">
+        <is>
+          <t>841.88 KB</t>
+        </is>
+      </c>
+      <c r="G29" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:19</t>
+        </is>
+      </c>
+      <c r="H29" s="8" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs/036_Governance andDisaster Management A Study ofSikkim.pdf</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>036_Governance andDisaster Management A Study ofSikkim</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>PDF Document</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t>.pdf</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>2.80 MB</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:19</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs/037_Traditional knowledge ondisaster management A preliminary study of the Lepcha co.pdf</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>037_Traditional knowledge ondisaster management A preliminary study of the Lepcha co</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>PDF Document</t>
+        </is>
+      </c>
+      <c r="E31" s="9" t="inlineStr">
+        <is>
+          <t>.pdf</t>
+        </is>
+      </c>
+      <c r="F31" s="9" t="inlineStr">
+        <is>
+          <t>114.89 KB</t>
+        </is>
+      </c>
+      <c r="G31" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:19</t>
+        </is>
+      </c>
+      <c r="H31" s="8" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs/039_Challenges indisaster Managementin Hill areas A Case Study ofSikkim.pdf</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>039_Challenges indisaster Managementin Hill areas A Case Study ofSikkim</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>PDF Document</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
+        <is>
+          <t>.pdf</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>5.53 MB</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:19</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="7" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs/041_UrbanWater Policyin the Eastern Himalayan State ofSikkim An Assessment.pdf</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>041_UrbanWater Policyin the Eastern Himalayan State ofSikkim An Assessment</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>PDF Document</t>
+        </is>
+      </c>
+      <c r="E33" s="9" t="inlineStr">
+        <is>
+          <t>.pdf</t>
+        </is>
+      </c>
+      <c r="F33" s="9" t="inlineStr">
+        <is>
+          <t>152.55 KB</t>
+        </is>
+      </c>
+      <c r="G33" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:19</t>
+        </is>
+      </c>
+      <c r="H33" s="8" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs/042_Water Resource Managementin SouthSikkim Community Participation and Institutiona.pdf</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>042_Water Resource Managementin SouthSikkim Community Participation and Institutiona</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>PDF Document</t>
+        </is>
+      </c>
+      <c r="E34" s="6" t="inlineStr">
+        <is>
+          <t>.pdf</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>4.54 MB</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:19</t>
+        </is>
+      </c>
+      <c r="H34" s="5" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="7" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs/043_[B]Ruralenergyplanning inSikkim.pdf</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>043_[B]Ruralenergyplanning inSikkim</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>PDF Document</t>
+        </is>
+      </c>
+      <c r="E35" s="9" t="inlineStr">
+        <is>
+          <t>.pdf</t>
+        </is>
+      </c>
+      <c r="F35" s="9" t="inlineStr">
+        <is>
+          <t>9.15 MB</t>
+        </is>
+      </c>
+      <c r="G35" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:19</t>
+        </is>
+      </c>
+      <c r="H35" s="8" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs/046_[B]Sikkim.pdf</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>046_[B]Sikkim</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>PDF Document</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>.pdf</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>10.84 MB</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:19</t>
+        </is>
+      </c>
+      <c r="H36" s="5" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="7" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs/047_Tourism inSikkim quest for a self-reliant economy.pdf</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>047_Tourism inSikkim quest for a self-reliant economy</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>PDF Document</t>
+        </is>
+      </c>
+      <c r="E37" s="9" t="inlineStr">
+        <is>
+          <t>.pdf</t>
+        </is>
+      </c>
+      <c r="F37" s="9" t="inlineStr">
+        <is>
+          <t>263.04 KB</t>
+        </is>
+      </c>
+      <c r="G37" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:19</t>
+        </is>
+      </c>
+      <c r="H37" s="8" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs/048_Agro-Economic environment andfoodsecurity inSikkim.pdf</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>048_Agro-Economic environment andfoodsecurity inSikkim</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>PDF Document</t>
+        </is>
+      </c>
+      <c r="E38" s="6" t="inlineStr">
+        <is>
+          <t>.pdf</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="inlineStr">
+        <is>
+          <t>8.76 MB</t>
+        </is>
+      </c>
+      <c r="G38" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:20</t>
+        </is>
+      </c>
+      <c r="H38" s="5" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="7" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="8" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs/049_Economic Evaluation of Farmer Producer Organisations inSikkim.pdf</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>049_Economic Evaluation of Farmer Producer Organisations inSikkim</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>PDF Document</t>
+        </is>
+      </c>
+      <c r="E39" s="9" t="inlineStr">
+        <is>
+          <t>.pdf</t>
+        </is>
+      </c>
+      <c r="F39" s="9" t="inlineStr">
+        <is>
+          <t>10.76 MB</t>
+        </is>
+      </c>
+      <c r="G39" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:20</t>
+        </is>
+      </c>
+      <c r="H39" s="8" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs/050_[B]UnderstandingFoodSecurity inSikkim A Case Study of Tathanchen Shyari Ward.pdf</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>050_[B]UnderstandingFoodSecurity inSikkim A Case Study of Tathanchen Shyari Ward</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>PDF Document</t>
+        </is>
+      </c>
+      <c r="E40" s="6" t="inlineStr">
+        <is>
+          <t>.pdf</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="inlineStr">
+        <is>
+          <t>4.95 MB</t>
+        </is>
+      </c>
+      <c r="G40" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:19</t>
+        </is>
+      </c>
+      <c r="H40" s="5" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="8" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs/051_A Critical Review ofFoodSecurity inSikkim.pdf</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>051_A Critical Review ofFoodSecurity inSikkim</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>PDF Document</t>
+        </is>
+      </c>
+      <c r="E41" s="9" t="inlineStr">
+        <is>
+          <t>.pdf</t>
+        </is>
+      </c>
+      <c r="F41" s="9" t="inlineStr">
+        <is>
+          <t>1.61 MB</t>
+        </is>
+      </c>
+      <c r="G41" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:19</t>
+        </is>
+      </c>
+      <c r="H41" s="8" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs/052_Sikkim.pdf</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>052_Sikkim</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>PDF Document</t>
+        </is>
+      </c>
+      <c r="E42" s="6" t="inlineStr">
+        <is>
+          <t>.pdf</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="inlineStr">
+        <is>
+          <t>4.05 MB</t>
+        </is>
+      </c>
+      <c r="G42" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:19</t>
+        </is>
+      </c>
+      <c r="H42" s="5" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="7" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="8" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs/053_GreenInvestments as a Vital Tool to Maintain the Sustainability of Tourist Desti.pdf</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>053_GreenInvestments as a Vital Tool to Maintain the Sustainability of Tourist Desti</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>PDF Document</t>
+        </is>
+      </c>
+      <c r="E43" s="9" t="inlineStr">
+        <is>
+          <t>.pdf</t>
+        </is>
+      </c>
+      <c r="F43" s="9" t="inlineStr">
+        <is>
+          <t>246.87 KB</t>
+        </is>
+      </c>
+      <c r="G43" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:19</t>
+        </is>
+      </c>
+      <c r="H43" s="8" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="A44" s="3" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs/054_Economic History ofSikkim A Study of the Planned Economy, 1954-1971.pdf</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>054_Economic History ofSikkim A Study of the Planned Economy, 1954-1971</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>PDF Document</t>
+        </is>
+      </c>
+      <c r="E44" s="6" t="inlineStr">
+        <is>
+          <t>.pdf</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="inlineStr">
+        <is>
+          <t>3.00 MB</t>
+        </is>
+      </c>
+      <c r="G44" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:19</t>
+        </is>
+      </c>
+      <c r="H44" s="5" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="A45" s="7" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="8" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs/057_SikkimHuman.pdf</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>057_SikkimHuman</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>PDF Document</t>
+        </is>
+      </c>
+      <c r="E45" s="9" t="inlineStr">
+        <is>
+          <t>.pdf</t>
+        </is>
+      </c>
+      <c r="F45" s="9" t="inlineStr">
+        <is>
+          <t>1.37 MB</t>
+        </is>
+      </c>
+      <c r="G45" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:19</t>
+        </is>
+      </c>
+      <c r="H45" s="8" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="A46" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs/058_Economy and social development of ruralSikkim.pdf</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>058_Economy and social development of ruralSikkim</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>PDF Document</t>
+        </is>
+      </c>
+      <c r="E46" s="6" t="inlineStr">
+        <is>
+          <t>.pdf</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="inlineStr">
+        <is>
+          <t>2.57 MB</t>
+        </is>
+      </c>
+      <c r="G46" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:19</t>
+        </is>
+      </c>
+      <c r="H46" s="5" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="20" customHeight="1">
+      <c r="A47" s="7" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="8" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs/060_Geospatial analysis of Socio-Economic Health Gnathang Valley andSikkim-Himalayas.pdf</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>060_Geospatial analysis of Socio-Economic Health Gnathang Valley andSikkim-Himalayas</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>PDF Document</t>
+        </is>
+      </c>
+      <c r="E47" s="9" t="inlineStr">
+        <is>
+          <t>.pdf</t>
+        </is>
+      </c>
+      <c r="F47" s="9" t="inlineStr">
+        <is>
+          <t>5.68 MB</t>
+        </is>
+      </c>
+      <c r="G47" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:19</t>
+        </is>
+      </c>
+      <c r="H47" s="8" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="20" customHeight="1">
+      <c r="A48" s="3" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs/061_[B]Sikkim the Story of its Integration with India.pdf</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>061_[B]Sikkim the Story of its Integration with India</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>PDF Document</t>
+        </is>
+      </c>
+      <c r="E48" s="6" t="inlineStr">
+        <is>
+          <t>.pdf</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="inlineStr">
+        <is>
+          <t>10.08 MB</t>
+        </is>
+      </c>
+      <c r="G48" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:19</t>
+        </is>
+      </c>
+      <c r="H48" s="5" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="20" customHeight="1">
+      <c r="A49" s="7" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="8" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs/063_Reducing the VulneRability of the PooR by buildingResilience a case study fRom s.pdf</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>063_Reducing the VulneRability of the PooR by buildingResilience a case study fRom s</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>PDF Document</t>
+        </is>
+      </c>
+      <c r="E49" s="9" t="inlineStr">
+        <is>
+          <t>.pdf</t>
+        </is>
+      </c>
+      <c r="F49" s="9" t="inlineStr">
+        <is>
+          <t>2.95 MB</t>
+        </is>
+      </c>
+      <c r="G49" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:19</t>
+        </is>
+      </c>
+      <c r="H49" s="8" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="20" customHeight="1">
+      <c r="A50" s="3" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs/064_MeasuringResilienceto Climate Change inSikkim Developing a ClimateResilienceInde.pdf</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>064_MeasuringResilienceto Climate Change inSikkim Developing a ClimateResilienceInde</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>PDF Document</t>
+        </is>
+      </c>
+      <c r="E50" s="6" t="inlineStr">
+        <is>
+          <t>.pdf</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="inlineStr">
+        <is>
+          <t>661.28 KB</t>
+        </is>
+      </c>
+      <c r="G50" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:19</t>
+        </is>
+      </c>
+      <c r="H50" s="5" t="inlineStr">
+        <is>
+          <t>scraped_policy_pdfs</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="20" customHeight="1">
+      <c r="A51" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="8" t="inlineStr">
+        <is>
+          <t>scraping.py</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>scraping</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>Python Source Code</t>
+        </is>
+      </c>
+      <c r="E51" s="9" t="inlineStr">
+        <is>
+          <t>.py</t>
+        </is>
+      </c>
+      <c r="F51" s="9" t="inlineStr">
+        <is>
+          <t>19.33 KB</t>
+        </is>
+      </c>
+      <c r="G51" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-19 12:58</t>
+        </is>
+      </c>
+      <c r="H51" s="8" t="inlineStr">
+        <is>
+          <t>Project Root</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="20" customHeight="1">
+      <c r="A52" s="3" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>requirements.txt</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>requirements</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Text Document</t>
+        </is>
+      </c>
+      <c r="E52" s="6" t="inlineStr">
+        <is>
+          <t>.txt</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="inlineStr">
+        <is>
+          <t>796 B</t>
+        </is>
+      </c>
+      <c r="G52" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-19 15:56</t>
+        </is>
+      </c>
+      <c r="H52" s="5" t="inlineStr">
+        <is>
+          <t>Project Root</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="20" customHeight="1">
+      <c r="A53" s="7" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="8" t="inlineStr">
+        <is>
+          <t>.gitignore</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>.gitignore</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>Configuration File</t>
+        </is>
+      </c>
+      <c r="E53" s="9" t="inlineStr"/>
+      <c r="F53" s="9" t="inlineStr">
+        <is>
+          <t>146 B</t>
+        </is>
+      </c>
+      <c r="G53" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:08</t>
+        </is>
+      </c>
+      <c r="H53" s="8" t="inlineStr">
+        <is>
+          <t>Project Root</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="20" customHeight="1">
+      <c r="A54" s="3" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
           <t>README.md</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C54" s="5" t="inlineStr">
         <is>
           <t>README</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
+      <c r="D54" s="5" t="inlineStr">
         <is>
           <t>Markdown Document</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr">
+      <c r="E54" s="6" t="inlineStr">
         <is>
           <t>.md</t>
         </is>
       </c>
-      <c r="F11" s="9" t="inlineStr">
-        <is>
-          <t>22 B</t>
-        </is>
-      </c>
-      <c r="G11" s="9" t="inlineStr">
-        <is>
-          <t>2026-05-19 14:10</t>
-        </is>
-      </c>
-      <c r="H11" s="8" t="inlineStr">
+      <c r="F54" s="6" t="inlineStr">
+        <is>
+          <t>2.44 KB</t>
+        </is>
+      </c>
+      <c r="G54" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-19 15:56</t>
+        </is>
+      </c>
+      <c r="H54" s="5" t="inlineStr">
         <is>
           <t>Project Root</t>
         </is>

</xml_diff>

<commit_message>
Implement incremental Excel indexing and download skipping
</commit_message>
<xml_diff>
--- a/scraped_results/sikkim_policy_files_index.xlsx
+++ b/scraped_results/sikkim_policy_files_index.xlsx
@@ -581,7 +581,7 @@
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>2026-05-19 12:13</t>
+          <t>2026-05-19 16:48</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
@@ -621,7 +621,7 @@
       </c>
       <c r="G3" s="8" t="inlineStr">
         <is>
-          <t>2026-05-19 12:13</t>
+          <t>2026-05-19 16:47</t>
         </is>
       </c>
       <c r="H3" s="7" t="inlineStr">
@@ -661,7 +661,7 @@
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>2026-05-19 12:04</t>
+          <t>2026-05-19 16:48</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
@@ -701,7 +701,7 @@
       </c>
       <c r="G5" s="8" t="inlineStr">
         <is>
-          <t>2026-05-19 11:45</t>
+          <t>2026-05-19 16:48</t>
         </is>
       </c>
       <c r="H5" s="7" t="inlineStr">
@@ -741,7 +741,7 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>2026-05-19 12:12</t>
+          <t>2026-05-19 16:48</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
@@ -781,7 +781,7 @@
       </c>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>2026-05-19 12:04</t>
+          <t>2026-05-19 16:48</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr">

</xml_diff>